<commit_message>
Merge remote main into desktop Chapter 2 changes
</commit_message>
<xml_diff>
--- a/chapter_1/results/enrichment/ora/ORA_exp1_combined_nested_semantic_calculating for results.xlsx
+++ b/chapter_1/results/enrichment/ora/ORA_exp1_combined_nested_semantic_calculating for results.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hamis\OneDrive\Documents\PhD\PhD---omics-analysis-portfolio\Chapter 1\Results\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/980ed44706d46718/Documents/PhD/PhD---omics-analysis-portfolio/chapter_1/results/enrichment/ora/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{109B395F-3E81-40E1-ACBD-0118D358A86B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="8_{109B395F-3E81-40E1-ACBD-0118D358A86B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AD4DB366-95DF-413A-9C2C-408C29E0B71E}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{C6F4A34B-F9DE-4412-96A4-16A0C34228C8}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C6F4A34B-F9DE-4412-96A4-16A0C34228C8}"/>
   </bookViews>
   <sheets>
     <sheet name="ORA_exp1_combined_nested_semant" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,20 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">ORA_exp1_combined_nested_semant!$A$1:$M$83</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -1857,18 +1870,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22367674-FF78-4117-A5FB-FA17B2099A98}">
   <dimension ref="A1:M83"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="0" hidden="1" customWidth="1"/>
     <col min="3" max="3" width="75" bestFit="1" customWidth="1"/>
     <col min="4" max="10" width="0" hidden="1" customWidth="1"/>
-    <col min="11" max="11" width="20" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="21.42578125" customWidth="1"/>
-    <col min="13" max="13" width="68.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="19.44140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="106.21875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="68.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1909,7 +1922,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>170</v>
       </c>
@@ -1950,7 +1963,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>19</v>
       </c>
@@ -1991,7 +2004,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>26</v>
       </c>
@@ -2032,7 +2045,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>203</v>
       </c>
@@ -2073,7 +2086,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>35</v>
       </c>
@@ -2114,7 +2127,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>40</v>
       </c>
@@ -2155,7 +2168,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>44</v>
       </c>
@@ -2196,7 +2209,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>48</v>
       </c>
@@ -2238,7 +2251,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>52</v>
       </c>
@@ -2279,7 +2292,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>57</v>
       </c>
@@ -2320,7 +2333,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>61</v>
       </c>
@@ -2361,7 +2374,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>65</v>
       </c>
@@ -2403,7 +2416,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>67</v>
       </c>
@@ -2444,7 +2457,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>70</v>
       </c>
@@ -2485,7 +2498,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>74</v>
       </c>
@@ -2526,7 +2539,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>79</v>
       </c>
@@ -2567,7 +2580,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>83</v>
       </c>
@@ -2608,7 +2621,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>311</v>
       </c>
@@ -2649,7 +2662,7 @@
         <v>313</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>278</v>
       </c>
@@ -2690,7 +2703,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>126</v>
       </c>
@@ -2731,7 +2744,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>306</v>
       </c>
@@ -2772,7 +2785,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>214</v>
       </c>
@@ -2813,7 +2826,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>223</v>
       </c>
@@ -2854,7 +2867,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>122</v>
       </c>
@@ -2895,7 +2908,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>167</v>
       </c>
@@ -2936,7 +2949,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>93</v>
       </c>
@@ -2977,7 +2990,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>231</v>
       </c>
@@ -3018,7 +3031,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>177</v>
       </c>
@@ -3059,7 +3072,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>130</v>
       </c>
@@ -3101,7 +3114,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>134</v>
       </c>
@@ -3142,7 +3155,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>173</v>
       </c>
@@ -3183,7 +3196,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>142</v>
       </c>
@@ -3224,7 +3237,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>145</v>
       </c>
@@ -3265,7 +3278,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>157</v>
       </c>
@@ -3306,7 +3319,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>296</v>
       </c>
@@ -3348,7 +3361,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>164</v>
       </c>
@@ -3389,7 +3402,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>160</v>
       </c>
@@ -3430,7 +3443,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>266</v>
       </c>
@@ -3471,7 +3484,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>308</v>
       </c>
@@ -3512,7 +3525,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>113</v>
       </c>
@@ -3553,7 +3566,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>261</v>
       </c>
@@ -3594,7 +3607,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>318</v>
       </c>
@@ -3635,7 +3648,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>181</v>
       </c>
@@ -3676,7 +3689,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>186</v>
       </c>
@@ -3717,7 +3730,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>191</v>
       </c>
@@ -3758,7 +3771,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>195</v>
       </c>
@@ -3799,7 +3812,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>198</v>
       </c>
@@ -3840,7 +3853,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>30</v>
       </c>
@@ -3881,7 +3894,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="50" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>207</v>
       </c>
@@ -3922,7 +3935,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="51" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>211</v>
       </c>
@@ -3963,7 +3976,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="52" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>235</v>
       </c>
@@ -4004,7 +4017,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="53" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>218</v>
       </c>
@@ -4045,7 +4058,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="54" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>118</v>
       </c>
@@ -4086,7 +4099,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="55" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>226</v>
       </c>
@@ -4127,7 +4140,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="56" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>229</v>
       </c>
@@ -4168,7 +4181,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="57" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>153</v>
       </c>
@@ -4209,7 +4222,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="58" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>13</v>
       </c>
@@ -4250,7 +4263,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="59" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>289</v>
       </c>
@@ -4291,7 +4304,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="60" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>87</v>
       </c>
@@ -4332,7 +4345,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="61" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>91</v>
       </c>
@@ -4373,7 +4386,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="62" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>300</v>
       </c>
@@ -4414,7 +4427,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="63" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>252</v>
       </c>
@@ -4455,7 +4468,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="64" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>257</v>
       </c>
@@ -4497,7 +4510,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="65" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>241</v>
       </c>
@@ -4538,7 +4551,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="66" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>269</v>
       </c>
@@ -4579,7 +4592,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="67" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>149</v>
       </c>
@@ -4620,7 +4633,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="68" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>103</v>
       </c>
@@ -4661,7 +4674,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="69" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>273</v>
       </c>
@@ -4702,7 +4715,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="70" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>106</v>
       </c>
@@ -4743,7 +4756,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="71" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>292</v>
       </c>
@@ -4785,7 +4798,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="72" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>286</v>
       </c>
@@ -4826,7 +4839,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="73" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>98</v>
       </c>
@@ -4867,7 +4880,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="74" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>321</v>
       </c>
@@ -4908,7 +4921,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="75" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>238</v>
       </c>
@@ -4949,7 +4962,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="76" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>244</v>
       </c>
@@ -4990,7 +5003,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="77" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>303</v>
       </c>
@@ -5031,7 +5044,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="78" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>282</v>
       </c>
@@ -5072,7 +5085,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="79" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>247</v>
       </c>
@@ -5113,7 +5126,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="80" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>108</v>
       </c>
@@ -5154,7 +5167,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="81" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>314</v>
       </c>
@@ -5195,7 +5208,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="82" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>138</v>
       </c>
@@ -5236,7 +5249,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="83" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>264</v>
       </c>

</xml_diff>